<commit_message>
fix(campo):Modifica nombre campo TIPO_MOV_DESCRI
</commit_message>
<xml_diff>
--- a/Movimientos_Circular_011_extraidos.xlsx
+++ b/Movimientos_Circular_011_extraidos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalhitss-my.sharepoint.com/personal/lozanoaa_hitss_com/Documents/Documentos Personales/Trabajos Freelance/Macro_Marlon/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Fuentes_Personales\Ciruclar_011\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_8A467017D7A0F843FDD5DD35A6B33C0357712905" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED8C01F6-D8BC-4854-9A2B-FC2C9050F3CF}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{168DFB8D-2DBF-4DB3-97C0-CC2362D805D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -53,9 +53,6 @@
     <t>TIPO_MOV</t>
   </si>
   <si>
-    <t>TIPO_MOV_DESC</t>
-  </si>
-  <si>
     <t>OFICINA</t>
   </si>
   <si>
@@ -198,6 +195,9 @@
   </si>
   <si>
     <t>Se transcribieron los datos que se distinguen con suficiente claridad. Las zonas afectadas por reflejos/moiré o baja resolución pueden requerir validación contra el archivo Excel original.</t>
+  </si>
+  <si>
+    <t>TIPO_MOV_DESCRI</t>
   </si>
 </sst>
 </file>
@@ -578,14 +578,15 @@
     <col min="2" max="2" width="42" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="33" customWidth="1"/>
-    <col min="5" max="6" width="12" customWidth="1"/>
+    <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="32" customWidth="1"/>
-    <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="8" max="8" width="34.140625" customWidth="1"/>
+    <col min="9" max="9" width="22.85546875" customWidth="1"/>
     <col min="10" max="10" width="42" customWidth="1"/>
-    <col min="11" max="11" width="12" customWidth="1"/>
+    <col min="11" max="11" width="13" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="21" customWidth="1"/>
-    <col min="13" max="13" width="14" customWidth="1"/>
+    <col min="13" max="13" width="19.5703125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="13" customWidth="1"/>
   </cols>
   <sheetData>
@@ -618,19 +619,19 @@
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -638,22 +639,22 @@
         <v>60</v>
       </c>
       <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>15</v>
-      </c>
       <c r="D2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
         <v>16</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>17</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>18</v>
-      </c>
-      <c r="G2" t="s">
-        <v>19</v>
       </c>
       <c r="H2" s="2">
         <v>590023221</v>
@@ -662,16 +663,16 @@
         <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K2">
         <v>1</v>
       </c>
       <c r="L2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N2" s="3">
         <v>1000000</v>
@@ -682,22 +683,22 @@
         <v>60</v>
       </c>
       <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
         <v>14</v>
       </c>
-      <c r="C3" t="s">
-        <v>15</v>
-      </c>
       <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
         <v>16</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>17</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>18</v>
-      </c>
-      <c r="G3" t="s">
-        <v>19</v>
       </c>
       <c r="H3" s="2">
         <v>590027705</v>
@@ -706,16 +707,16 @@
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K3">
         <v>1</v>
       </c>
       <c r="L3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N3" s="3">
         <v>1586366</v>
@@ -726,22 +727,22 @@
         <v>60</v>
       </c>
       <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
         <v>14</v>
       </c>
-      <c r="C4" t="s">
-        <v>15</v>
-      </c>
       <c r="D4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" t="s">
         <v>16</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>17</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>18</v>
-      </c>
-      <c r="G4" t="s">
-        <v>19</v>
       </c>
       <c r="H4" s="2">
         <v>590028126</v>
@@ -750,16 +751,16 @@
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K4">
         <v>1</v>
       </c>
       <c r="L4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N4" s="3">
         <v>18000</v>
@@ -770,22 +771,22 @@
         <v>60</v>
       </c>
       <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
         <v>14</v>
       </c>
-      <c r="C5" t="s">
-        <v>15</v>
-      </c>
       <c r="D5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" t="s">
         <v>16</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>17</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>18</v>
-      </c>
-      <c r="G5" t="s">
-        <v>19</v>
       </c>
       <c r="H5" s="2">
         <v>590028130</v>
@@ -794,16 +795,16 @@
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K5">
         <v>1</v>
       </c>
       <c r="L5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N5" s="3">
         <v>4666518</v>
@@ -814,22 +815,22 @@
         <v>60</v>
       </c>
       <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
         <v>14</v>
       </c>
-      <c r="C6" t="s">
-        <v>15</v>
-      </c>
       <c r="D6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" t="s">
         <v>16</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>17</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>18</v>
-      </c>
-      <c r="G6" t="s">
-        <v>19</v>
       </c>
       <c r="H6" s="2">
         <v>590028391</v>
@@ -838,16 +839,16 @@
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K6">
         <v>1</v>
       </c>
       <c r="L6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N6" s="3">
         <v>18248757</v>
@@ -858,22 +859,22 @@
         <v>60</v>
       </c>
       <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
         <v>14</v>
       </c>
-      <c r="C7" t="s">
-        <v>15</v>
-      </c>
       <c r="D7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" t="s">
         <v>16</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>17</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>18</v>
-      </c>
-      <c r="G7" t="s">
-        <v>19</v>
       </c>
       <c r="H7" s="2">
         <v>590035860</v>
@@ -882,16 +883,16 @@
         <v>971</v>
       </c>
       <c r="J7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K7">
         <v>1</v>
       </c>
       <c r="L7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N7" s="3">
         <v>-1000000</v>
@@ -902,22 +903,22 @@
         <v>60</v>
       </c>
       <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" t="s">
         <v>14</v>
       </c>
-      <c r="C8" t="s">
-        <v>15</v>
-      </c>
       <c r="D8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" t="s">
         <v>16</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>17</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>18</v>
-      </c>
-      <c r="G8" t="s">
-        <v>19</v>
       </c>
       <c r="H8" s="2">
         <v>590035863</v>
@@ -926,16 +927,16 @@
         <v>973</v>
       </c>
       <c r="J8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K8">
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N8" s="3">
         <v>-8087</v>
@@ -946,22 +947,22 @@
         <v>60</v>
       </c>
       <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" t="s">
         <v>14</v>
       </c>
-      <c r="C9" t="s">
-        <v>15</v>
-      </c>
       <c r="D9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" t="s">
         <v>16</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>17</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>18</v>
-      </c>
-      <c r="G9" t="s">
-        <v>19</v>
       </c>
       <c r="H9" s="2">
         <v>590037483</v>
@@ -970,16 +971,16 @@
         <v>1</v>
       </c>
       <c r="J9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K9">
         <v>1</v>
       </c>
       <c r="L9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N9" s="3">
         <v>4600000</v>
@@ -990,22 +991,22 @@
         <v>60</v>
       </c>
       <c r="B10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" t="s">
         <v>14</v>
       </c>
-      <c r="C10" t="s">
-        <v>15</v>
-      </c>
       <c r="D10" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" t="s">
         <v>16</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>17</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>18</v>
-      </c>
-      <c r="G10" t="s">
-        <v>19</v>
       </c>
       <c r="H10" s="2">
         <v>590037490</v>
@@ -1014,16 +1015,16 @@
         <v>1</v>
       </c>
       <c r="J10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K10">
         <v>1</v>
       </c>
       <c r="L10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N10" s="3">
         <v>67000000</v>
@@ -1034,22 +1035,22 @@
         <v>60</v>
       </c>
       <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" t="s">
         <v>14</v>
       </c>
-      <c r="C11" t="s">
-        <v>15</v>
-      </c>
       <c r="D11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" t="s">
         <v>16</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>17</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>18</v>
-      </c>
-      <c r="G11" t="s">
-        <v>19</v>
       </c>
       <c r="H11" s="2">
         <v>590037527</v>
@@ -1058,16 +1059,16 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K11">
         <v>1</v>
       </c>
       <c r="L11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N11" s="3">
         <v>375170000</v>
@@ -1078,22 +1079,22 @@
         <v>60</v>
       </c>
       <c r="B12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" t="s">
         <v>14</v>
       </c>
-      <c r="C12" t="s">
-        <v>15</v>
-      </c>
       <c r="D12" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" t="s">
         <v>16</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>17</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>18</v>
-      </c>
-      <c r="G12" t="s">
-        <v>19</v>
       </c>
       <c r="H12" s="2">
         <v>590039519</v>
@@ -1102,16 +1103,16 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K12">
         <v>1</v>
       </c>
       <c r="L12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N12" s="3">
         <v>25784076</v>
@@ -1122,22 +1123,22 @@
         <v>60</v>
       </c>
       <c r="B13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" t="s">
         <v>14</v>
       </c>
-      <c r="C13" t="s">
-        <v>15</v>
-      </c>
       <c r="D13" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" t="s">
         <v>16</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>17</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>18</v>
-      </c>
-      <c r="G13" t="s">
-        <v>19</v>
       </c>
       <c r="H13" s="2">
         <v>590153436</v>
@@ -1146,16 +1147,16 @@
         <v>130</v>
       </c>
       <c r="J13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K13">
         <v>1</v>
       </c>
       <c r="L13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N13" s="3">
         <v>2958570</v>
@@ -1166,22 +1167,22 @@
         <v>60</v>
       </c>
       <c r="B14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" t="s">
         <v>14</v>
       </c>
-      <c r="C14" t="s">
-        <v>15</v>
-      </c>
       <c r="D14" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" t="s">
         <v>16</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>17</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>18</v>
-      </c>
-      <c r="G14" t="s">
-        <v>19</v>
       </c>
       <c r="H14" s="2">
         <v>590153437</v>
@@ -1190,16 +1191,16 @@
         <v>90</v>
       </c>
       <c r="J14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K14">
         <v>1</v>
       </c>
       <c r="L14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N14" s="3">
         <v>-54571763</v>
@@ -1210,22 +1211,22 @@
         <v>60</v>
       </c>
       <c r="B15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" t="s">
         <v>14</v>
       </c>
-      <c r="C15" t="s">
-        <v>15</v>
-      </c>
       <c r="D15" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15" t="s">
         <v>16</v>
       </c>
-      <c r="E15" t="s">
-        <v>17</v>
-      </c>
       <c r="F15" t="s">
+        <v>26</v>
+      </c>
+      <c r="G15" t="s">
         <v>27</v>
-      </c>
-      <c r="G15" t="s">
-        <v>28</v>
       </c>
       <c r="H15" s="2">
         <v>590194988</v>
@@ -1234,16 +1235,16 @@
         <v>44</v>
       </c>
       <c r="J15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K15">
         <v>1</v>
       </c>
       <c r="L15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N15" s="3">
         <v>-130000000</v>
@@ -1254,22 +1255,22 @@
         <v>60</v>
       </c>
       <c r="B16" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" t="s">
         <v>14</v>
       </c>
-      <c r="C16" t="s">
-        <v>15</v>
-      </c>
       <c r="D16" t="s">
+        <v>15</v>
+      </c>
+      <c r="E16" t="s">
         <v>16</v>
       </c>
-      <c r="E16" t="s">
-        <v>17</v>
-      </c>
       <c r="F16" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" t="s">
         <v>27</v>
-      </c>
-      <c r="G16" t="s">
-        <v>28</v>
       </c>
       <c r="H16" s="2">
         <v>590194989</v>
@@ -1278,16 +1279,16 @@
         <v>45</v>
       </c>
       <c r="J16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K16">
         <v>1</v>
       </c>
       <c r="L16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N16" s="3">
         <v>54571763830</v>
@@ -1298,22 +1299,22 @@
         <v>109</v>
       </c>
       <c r="B17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" t="s">
         <v>31</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
+        <v>15</v>
+      </c>
+      <c r="E17" t="s">
         <v>32</v>
       </c>
-      <c r="D17" t="s">
-        <v>16</v>
-      </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>33</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>34</v>
-      </c>
-      <c r="G17" t="s">
-        <v>35</v>
       </c>
       <c r="H17" s="2">
         <v>89086079</v>
@@ -1322,16 +1323,16 @@
         <v>971</v>
       </c>
       <c r="J17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K17">
         <v>3836</v>
       </c>
       <c r="L17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M17" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N17" s="3">
         <v>-227874</v>
@@ -1342,22 +1343,22 @@
         <v>109</v>
       </c>
       <c r="B18" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" t="s">
         <v>31</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
+        <v>15</v>
+      </c>
+      <c r="E18" t="s">
         <v>32</v>
       </c>
-      <c r="D18" t="s">
-        <v>16</v>
-      </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>33</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>34</v>
-      </c>
-      <c r="G18" t="s">
-        <v>35</v>
       </c>
       <c r="H18" s="2">
         <v>89086081</v>
@@ -1366,16 +1367,16 @@
         <v>973</v>
       </c>
       <c r="J18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K18">
         <v>3836</v>
       </c>
       <c r="L18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N18" s="3">
         <v>789258</v>
@@ -1386,22 +1387,22 @@
         <v>109</v>
       </c>
       <c r="B19" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19" t="s">
         <v>31</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
+        <v>15</v>
+      </c>
+      <c r="E19" t="s">
         <v>32</v>
       </c>
-      <c r="D19" t="s">
-        <v>16</v>
-      </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>33</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>34</v>
-      </c>
-      <c r="G19" t="s">
-        <v>35</v>
       </c>
       <c r="H19" s="2">
         <v>89086092</v>
@@ -1410,16 +1411,16 @@
         <v>971</v>
       </c>
       <c r="J19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K19">
         <v>3836</v>
       </c>
       <c r="L19" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N19" s="3">
         <v>-287651</v>
@@ -1430,22 +1431,22 @@
         <v>109</v>
       </c>
       <c r="B20" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" t="s">
         <v>31</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
+        <v>15</v>
+      </c>
+      <c r="E20" t="s">
         <v>32</v>
       </c>
-      <c r="D20" t="s">
-        <v>16</v>
-      </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>33</v>
       </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>34</v>
-      </c>
-      <c r="G20" t="s">
-        <v>35</v>
       </c>
       <c r="H20" s="2">
         <v>89086094</v>
@@ -1454,16 +1455,16 @@
         <v>973</v>
       </c>
       <c r="J20" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K20">
         <v>3836</v>
       </c>
       <c r="L20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N20" s="3">
         <v>-58932</v>
@@ -1474,22 +1475,22 @@
         <v>109</v>
       </c>
       <c r="B21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" t="s">
         <v>31</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
+        <v>15</v>
+      </c>
+      <c r="E21" t="s">
         <v>32</v>
       </c>
-      <c r="D21" t="s">
-        <v>16</v>
-      </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>33</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>34</v>
-      </c>
-      <c r="G21" t="s">
-        <v>35</v>
       </c>
       <c r="H21" s="2">
         <v>89086180</v>
@@ -1498,16 +1499,16 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K21">
         <v>3836</v>
       </c>
       <c r="L21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N21" s="3">
         <v>1781293</v>
@@ -1518,22 +1519,22 @@
         <v>109</v>
       </c>
       <c r="B22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22" t="s">
         <v>31</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
+        <v>15</v>
+      </c>
+      <c r="E22" t="s">
         <v>32</v>
       </c>
-      <c r="D22" t="s">
-        <v>16</v>
-      </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>33</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>34</v>
-      </c>
-      <c r="G22" t="s">
-        <v>35</v>
       </c>
       <c r="H22" s="2">
         <v>89098034</v>
@@ -1542,16 +1543,16 @@
         <v>130</v>
       </c>
       <c r="J22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K22">
         <v>3836</v>
       </c>
       <c r="L22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N22" s="3">
         <v>135246</v>
@@ -1562,22 +1563,22 @@
         <v>109</v>
       </c>
       <c r="B23" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23" t="s">
         <v>31</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
+        <v>15</v>
+      </c>
+      <c r="E23" t="s">
         <v>32</v>
       </c>
-      <c r="D23" t="s">
-        <v>16</v>
-      </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
         <v>33</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>34</v>
-      </c>
-      <c r="G23" t="s">
-        <v>35</v>
       </c>
       <c r="H23" s="2">
         <v>89098035</v>
@@ -1586,16 +1587,16 @@
         <v>90</v>
       </c>
       <c r="J23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K23">
         <v>3836</v>
       </c>
       <c r="L23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N23" s="3">
         <v>-2</v>
@@ -1606,22 +1607,22 @@
         <v>19</v>
       </c>
       <c r="B24" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" t="s">
         <v>36</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
+        <v>15</v>
+      </c>
+      <c r="E24" t="s">
         <v>37</v>
       </c>
-      <c r="D24" t="s">
-        <v>16</v>
-      </c>
-      <c r="E24" t="s">
+      <c r="F24" t="s">
         <v>38</v>
       </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>39</v>
-      </c>
-      <c r="G24" t="s">
-        <v>40</v>
       </c>
       <c r="H24" s="2">
         <v>4905553</v>
@@ -1630,16 +1631,16 @@
         <v>131</v>
       </c>
       <c r="J24" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K24">
         <v>3836</v>
       </c>
       <c r="L24" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N24" s="3">
         <v>-448</v>
@@ -1650,22 +1651,22 @@
         <v>191</v>
       </c>
       <c r="B25" t="s">
+        <v>41</v>
+      </c>
+      <c r="C25" t="s">
         <v>42</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
+        <v>15</v>
+      </c>
+      <c r="E25" t="s">
         <v>43</v>
       </c>
-      <c r="D25" t="s">
-        <v>16</v>
-      </c>
-      <c r="E25" t="s">
+      <c r="F25" t="s">
         <v>44</v>
       </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
         <v>45</v>
-      </c>
-      <c r="G25" t="s">
-        <v>46</v>
       </c>
       <c r="H25" s="2">
         <v>7227641</v>
@@ -1674,16 +1675,16 @@
         <v>131</v>
       </c>
       <c r="J25" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K25">
         <v>3836</v>
       </c>
       <c r="L25" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M25" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N25" s="3">
         <v>-150000</v>
@@ -1694,22 +1695,22 @@
         <v>700</v>
       </c>
       <c r="B26" t="s">
+        <v>46</v>
+      </c>
+      <c r="C26" t="s">
         <v>47</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>48</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>49</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26" t="s">
         <v>50</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>51</v>
-      </c>
-      <c r="G26" t="s">
-        <v>52</v>
       </c>
       <c r="H26" s="2">
         <v>7848743</v>
@@ -1718,16 +1719,16 @@
         <v>973</v>
       </c>
       <c r="J26" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K26">
         <v>3836</v>
       </c>
       <c r="L26" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M26" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N26" s="3">
         <v>-251369</v>
@@ -1738,22 +1739,22 @@
         <v>700</v>
       </c>
       <c r="B27" t="s">
+        <v>46</v>
+      </c>
+      <c r="C27" t="s">
         <v>47</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
         <v>48</v>
       </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
         <v>49</v>
       </c>
-      <c r="E27" t="s">
+      <c r="F27" t="s">
         <v>50</v>
       </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
         <v>51</v>
-      </c>
-      <c r="G27" t="s">
-        <v>52</v>
       </c>
       <c r="H27" s="2">
         <v>7848745</v>
@@ -1762,16 +1763,16 @@
         <v>973</v>
       </c>
       <c r="J27" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K27">
         <v>3836</v>
       </c>
       <c r="L27" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M27" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N27" s="3">
         <v>-1500000</v>
@@ -1782,22 +1783,22 @@
         <v>700</v>
       </c>
       <c r="B28" t="s">
+        <v>46</v>
+      </c>
+      <c r="C28" t="s">
         <v>47</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>48</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>49</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F28" t="s">
         <v>50</v>
       </c>
-      <c r="F28" t="s">
+      <c r="G28" t="s">
         <v>51</v>
-      </c>
-      <c r="G28" t="s">
-        <v>52</v>
       </c>
       <c r="H28" s="2">
         <v>7848749</v>
@@ -1806,16 +1807,16 @@
         <v>973</v>
       </c>
       <c r="J28" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K28">
         <v>3836</v>
       </c>
       <c r="L28" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M28" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N28" s="3">
         <v>-58932</v>
@@ -1826,22 +1827,22 @@
         <v>700</v>
       </c>
       <c r="B29" t="s">
+        <v>46</v>
+      </c>
+      <c r="C29" t="s">
         <v>47</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>48</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>49</v>
       </c>
-      <c r="E29" t="s">
+      <c r="F29" t="s">
         <v>50</v>
       </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>51</v>
-      </c>
-      <c r="G29" t="s">
-        <v>52</v>
       </c>
       <c r="H29" s="2">
         <v>7848753</v>
@@ -1850,16 +1851,16 @@
         <v>973</v>
       </c>
       <c r="J29" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K29">
         <v>3836</v>
       </c>
       <c r="L29" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M29" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N29" s="3">
         <v>-6587148</v>
@@ -1870,22 +1871,22 @@
         <v>700</v>
       </c>
       <c r="B30" t="s">
+        <v>46</v>
+      </c>
+      <c r="C30" t="s">
         <v>47</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>48</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>49</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F30" t="s">
         <v>50</v>
       </c>
-      <c r="F30" t="s">
+      <c r="G30" t="s">
         <v>51</v>
-      </c>
-      <c r="G30" t="s">
-        <v>52</v>
       </c>
       <c r="H30" s="2">
         <v>7848755</v>
@@ -1894,16 +1895,16 @@
         <v>973</v>
       </c>
       <c r="J30" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K30">
         <v>3836</v>
       </c>
       <c r="L30" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M30" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N30" s="3">
         <v>-89420</v>
@@ -1914,22 +1915,22 @@
         <v>700</v>
       </c>
       <c r="B31" t="s">
+        <v>46</v>
+      </c>
+      <c r="C31" t="s">
         <v>47</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>48</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>49</v>
       </c>
-      <c r="E31" t="s">
+      <c r="F31" t="s">
         <v>50</v>
       </c>
-      <c r="F31" t="s">
+      <c r="G31" t="s">
         <v>51</v>
-      </c>
-      <c r="G31" t="s">
-        <v>52</v>
       </c>
       <c r="H31" s="2">
         <v>7848757</v>
@@ -1938,16 +1939,16 @@
         <v>973</v>
       </c>
       <c r="J31" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K31">
         <v>3836</v>
       </c>
       <c r="L31" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M31" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N31" s="3">
         <v>-896863</v>
@@ -1958,22 +1959,22 @@
         <v>700</v>
       </c>
       <c r="B32" t="s">
+        <v>46</v>
+      </c>
+      <c r="C32" t="s">
         <v>47</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>48</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
         <v>49</v>
       </c>
-      <c r="E32" t="s">
+      <c r="F32" t="s">
         <v>50</v>
       </c>
-      <c r="F32" t="s">
+      <c r="G32" t="s">
         <v>51</v>
-      </c>
-      <c r="G32" t="s">
-        <v>52</v>
       </c>
       <c r="H32" s="2">
         <v>7848759</v>
@@ -1982,16 +1983,16 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K32">
         <v>3836</v>
       </c>
       <c r="L32" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M32" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N32" s="3">
         <v>400000000</v>
@@ -2002,22 +2003,22 @@
         <v>700</v>
       </c>
       <c r="B33" t="s">
+        <v>46</v>
+      </c>
+      <c r="C33" t="s">
         <v>47</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>48</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
         <v>49</v>
       </c>
-      <c r="E33" t="s">
+      <c r="F33" t="s">
         <v>50</v>
       </c>
-      <c r="F33" t="s">
+      <c r="G33" t="s">
         <v>51</v>
-      </c>
-      <c r="G33" t="s">
-        <v>52</v>
       </c>
       <c r="H33" s="2">
         <v>7849760</v>
@@ -2026,16 +2027,16 @@
         <v>130</v>
       </c>
       <c r="J33" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K33">
         <v>3836</v>
       </c>
       <c r="L33" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M33" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N33" s="3">
         <v>2871373</v>
@@ -2046,22 +2047,22 @@
         <v>700</v>
       </c>
       <c r="B34" t="s">
+        <v>46</v>
+      </c>
+      <c r="C34" t="s">
         <v>47</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>48</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
         <v>49</v>
       </c>
-      <c r="E34" t="s">
+      <c r="F34" t="s">
         <v>50</v>
       </c>
-      <c r="F34" t="s">
+      <c r="G34" t="s">
         <v>51</v>
-      </c>
-      <c r="G34" t="s">
-        <v>52</v>
       </c>
       <c r="H34" s="2">
         <v>7849761</v>
@@ -2070,16 +2071,16 @@
         <v>90</v>
       </c>
       <c r="J34" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K34">
         <v>3836</v>
       </c>
       <c r="L34" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M34" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N34" s="3">
         <v>78006</v>
@@ -2103,23 +2104,23 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" t="s">
         <v>54</v>
-      </c>
-      <c r="B2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>56</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>